<commit_message>
dashboard update added-have some bugs
</commit_message>
<xml_diff>
--- a/electron/data/summary_portfolio1.xlsx
+++ b/electron/data/summary_portfolio1.xlsx
@@ -475,16 +475,16 @@
         <v>384.2120704545454</v>
       </c>
       <c r="I2">
-        <v>449.88</v>
+        <v>444</v>
       </c>
       <c r="J2">
-        <v>-0.64</v>
+        <v>-6.52</v>
       </c>
       <c r="K2" t="str">
-        <v>(-0.14%)</v>
+        <v>(-1.45%)</v>
       </c>
       <c r="L2">
-        <v>17.09158420446436</v>
+        <v>15.561179396243835</v>
       </c>
       <c r="M2">
         <v>95.90637295493026</v>
@@ -522,16 +522,16 @@
         <v>18.0395</v>
       </c>
       <c r="I3">
-        <v>31.88</v>
+        <v>31.9</v>
       </c>
       <c r="J3">
-        <v>0.31</v>
+        <v>0.33</v>
       </c>
       <c r="K3" t="str">
-        <v>(0.98%)</v>
+        <v>(1.05%)</v>
       </c>
       <c r="L3">
-        <v>76.7233016436154</v>
+        <v>76.83416946145957</v>
       </c>
       <c r="M3">
         <v>4.0936270450697405</v>

</xml_diff>

<commit_message>
stats added but not implementation
</commit_message>
<xml_diff>
--- a/electron/data/summary_portfolio1.xlsx
+++ b/electron/data/summary_portfolio1.xlsx
@@ -472,16 +472,16 @@
         <v>400.695</v>
       </c>
       <c r="I2">
-        <v>444.8</v>
+        <v>444.99</v>
       </c>
       <c r="J2">
-        <v>-5.72</v>
+        <v>2.6</v>
       </c>
       <c r="K2" t="str">
-        <v>(-1.27%)</v>
+        <v>(0.59%)</v>
       </c>
       <c r="L2">
-        <v>11.007125120103824</v>
+        <v>11.05454273200315</v>
       </c>
       <c r="M2">
         <v>19.511868508719765</v>
@@ -519,16 +519,16 @@
         <v>25.048125</v>
       </c>
       <c r="I3">
-        <v>31.9</v>
+        <v>31.98</v>
       </c>
       <c r="J3">
-        <v>0.33</v>
+        <v>0.18</v>
       </c>
       <c r="K3" t="str">
-        <v>(1.05%)</v>
+        <v>(0.57%)</v>
       </c>
       <c r="L3">
-        <v>27.354841929286124</v>
+        <v>27.674227112807852</v>
       </c>
       <c r="M3">
         <v>12.197200399056046</v>
@@ -566,16 +566,16 @@
         <v>1402.42</v>
       </c>
       <c r="I4" t="str">
-        <v>1,912.88</v>
+        <v>1,939.00</v>
       </c>
       <c r="J4">
-        <v>-40.01</v>
+        <v>16.96</v>
       </c>
       <c r="K4" t="str">
-        <v>(-2.05%)</v>
+        <v>(0.88%)</v>
       </c>
       <c r="L4">
-        <v>36.39851114502075</v>
+        <v>38.2610059753854</v>
       </c>
       <c r="M4">
         <v>68.2909310922242</v>

</xml_diff>